<commit_message>
Fix canonical URL in sushi-config.yaml a70cdf695b7aabae44b083ef246caba763813f9a
</commit_message>
<xml_diff>
--- a/MAJSushiConfig/ig/CodeSystem-fr-cs-note-type.xlsx
+++ b/MAJSushiConfig/ig/CodeSystem-fr-cs-note-type.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/fhir-document-core/CodeSystem/fr-cs-note-type</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/document-core/CodeSystem/fr-cs-note-type</t>
   </si>
   <si>
     <t>Version</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-07T10:09:50+00:00</t>
+    <t>2026-09-07T10:25:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>